<commit_message>
DD counts paper plates; slice tray (G060510) counts like clamshells
James's July 6 confirmations:
- Paper plates count for Double Double too — platesCountForBrand is now
  "every brand except GINOS", the exclusion James actually stated.
- Ginos Pizza Slice Tray (G060510, 500/case) counts toward slice usage.
  The "Slice" in its description already routes it to the clamshell
  bucket, so mapping the product is the whole fix.

Verified against W15 2026: STORE 055 (DD) 2,720 -> 5,120 oz (+1,200
plates x 2 oz); GINOS002 10,280 -> 11,280 (+500 tray pieces x 2 oz);
GINOS103 and TTD ACTON unchanged. 54/54 tests pass.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/App Data.xlsx
+++ b/App Data.xlsx
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F38"/>
+  <dimension ref="A1:F39"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1166,10 +1166,30 @@
         <v>each</v>
       </c>
     </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>G060510</v>
+      </c>
+      <c r="B39" t="str">
+        <v>Ginos Pizza Slice Tray - 500/cs</v>
+      </c>
+      <c r="C39" t="str">
+        <v>Packaging</v>
+      </c>
+      <c r="D39" t="str">
+        <v>500/cs</v>
+      </c>
+      <c r="E39">
+        <v>500</v>
+      </c>
+      <c r="F39" t="str">
+        <v>each</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F38"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F39"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>